<commit_message>
fix: adjust sample excel data
</commit_message>
<xml_diff>
--- a/TurboVault_TPCH_Data.xlsx
+++ b/TurboVault_TPCH_Data.xlsx
@@ -979,7 +979,7 @@
         <v>SRC0004</v>
       </c>
       <c r="D3" t="str">
-        <v>C_CustomerKey</v>
+        <v>L_SUPPKEY</v>
       </c>
       <c r="E3" t="str">
         <v>C_CUSTKEY</v>
@@ -2786,7 +2786,7 @@
         <v>CUSTOMER_H</v>
       </c>
       <c r="G2" t="str">
-        <v>address_type</v>
+        <v>C_MKTSEGMENT</v>
       </c>
       <c r="H2" t="str">
         <v>customer_name</v>
@@ -2821,7 +2821,7 @@
         <v>CUSTOMER_H</v>
       </c>
       <c r="G3" t="str">
-        <v>address_type</v>
+        <v>C_MKTSEGMENT</v>
       </c>
       <c r="H3" t="str">
         <v>c_nationkey</v>
@@ -2853,7 +2853,7 @@
         <v>CUSTOMER_H</v>
       </c>
       <c r="G4" t="str">
-        <v>address_type</v>
+        <v>C_MKTSEGMENT</v>
       </c>
       <c r="I4" t="str">
         <v>3</v>
@@ -3521,7 +3521,7 @@
         <v>SRC0004</v>
       </c>
       <c r="D3" t="str">
-        <v>l_shipisntruct</v>
+        <v>l_shipinstruct</v>
       </c>
       <c r="E3" t="str">
         <v>NH0001</v>

</xml_diff>

<commit_message>
fix(excel-import): proper ref_table example
</commit_message>
<xml_diff>
--- a/TurboVault_TPCH_Data.xlsx
+++ b/TurboVault_TPCH_Data.xlsx
@@ -3613,7 +3613,7 @@
         <v>RS001</v>
       </c>
       <c r="E2" t="str">
-        <v>n_nationkey,r_regionkey</v>
+        <v>n_comment,n_regionkey</v>
       </c>
       <c r="G2" t="str">
         <v>latest</v>
@@ -3636,7 +3636,7 @@
         <v>RS002</v>
       </c>
       <c r="F3" t="str">
-        <v>n_nationkey,r_regionkey</v>
+        <v>n_comment,n_regionkey</v>
       </c>
       <c r="G3" t="str">
         <v>latest</v>

</xml_diff>

<commit_message>
Fully running dbt Project (#63)
- fix: dbt - adjust jinja templates to fix dbt models

- fix: adjust sample excel data

- fix: excel-import - avoid wrong prejoins

- fix: prejoins - add prejoined hub hashkeys to stage generations

- fix: excel-import - properly ingest reference table include & exclude columns

- fix: excel-import - proper ref_table example

- fix: ref-tables - fix json export for ref table include & exclude columns

- fix: ref-tables - added include & exclude columns to dbt model
</commit_message>
<xml_diff>
--- a/TurboVault_TPCH_Data.xlsx
+++ b/TurboVault_TPCH_Data.xlsx
@@ -979,7 +979,7 @@
         <v>SRC0004</v>
       </c>
       <c r="D3" t="str">
-        <v>C_CustomerKey</v>
+        <v>L_SUPPKEY</v>
       </c>
       <c r="E3" t="str">
         <v>C_CUSTKEY</v>
@@ -2786,7 +2786,7 @@
         <v>CUSTOMER_H</v>
       </c>
       <c r="G2" t="str">
-        <v>address_type</v>
+        <v>C_MKTSEGMENT</v>
       </c>
       <c r="H2" t="str">
         <v>customer_name</v>
@@ -2821,7 +2821,7 @@
         <v>CUSTOMER_H</v>
       </c>
       <c r="G3" t="str">
-        <v>address_type</v>
+        <v>C_MKTSEGMENT</v>
       </c>
       <c r="H3" t="str">
         <v>c_nationkey</v>
@@ -2853,7 +2853,7 @@
         <v>CUSTOMER_H</v>
       </c>
       <c r="G4" t="str">
-        <v>address_type</v>
+        <v>C_MKTSEGMENT</v>
       </c>
       <c r="I4" t="str">
         <v>3</v>
@@ -3521,7 +3521,7 @@
         <v>SRC0004</v>
       </c>
       <c r="D3" t="str">
-        <v>l_shipisntruct</v>
+        <v>l_shipinstruct</v>
       </c>
       <c r="E3" t="str">
         <v>NH0001</v>
@@ -3613,7 +3613,7 @@
         <v>RS001</v>
       </c>
       <c r="E2" t="str">
-        <v>n_nationkey,r_regionkey</v>
+        <v>n_comment,n_regionkey</v>
       </c>
       <c r="G2" t="str">
         <v>latest</v>
@@ -3636,7 +3636,7 @@
         <v>RS002</v>
       </c>
       <c r="F3" t="str">
-        <v>n_nationkey,r_regionkey</v>
+        <v>n_comment,n_regionkey</v>
       </c>
       <c r="G3" t="str">
         <v>latest</v>

</xml_diff>

<commit_message>
target_column_sort_order added to import and backend model
</commit_message>
<xml_diff>
--- a/TurboVault_TPCH_Data.xlsx
+++ b/TurboVault_TPCH_Data.xlsx
@@ -1968,7 +1968,7 @@
         <v>C_ACCTBAL</v>
       </c>
       <c r="H2" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2" t="str">
         <v>Customers</v>
@@ -2026,7 +2026,7 @@
         <v>C_COMMENT</v>
       </c>
       <c r="H4" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I4" t="str">
         <v>Customers</v>

</xml_diff>

<commit_message>
target_column_sort_order added to import and backend model (#118)
* target_column_sort_order added to import and backend model

* remove temp debug files
</commit_message>
<xml_diff>
--- a/TurboVault_TPCH_Data.xlsx
+++ b/TurboVault_TPCH_Data.xlsx
@@ -1968,7 +1968,7 @@
         <v>C_ACCTBAL</v>
       </c>
       <c r="H2" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2" t="str">
         <v>Customers</v>
@@ -2026,7 +2026,7 @@
         <v>C_COMMENT</v>
       </c>
       <c r="H4" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I4" t="str">
         <v>Customers</v>

</xml_diff>

<commit_message>
fix: generate effectivity satellite
</commit_message>
<xml_diff>
--- a/TurboVault_TPCH_Data.xlsx
+++ b/TurboVault_TPCH_Data.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="283">
   <si>
     <t>Pit_Identifier</t>
   </si>
@@ -762,6 +762,9 @@
   </si>
   <si>
     <t>Business_Key_Physical_Name</t>
+  </si>
+  <si>
+    <t>Effectivity_Satellite</t>
   </si>
   <si>
     <t>Is_Primary_Source</t>
@@ -877,13 +880,25 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -894,7 +909,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -906,13 +928,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1233,22 +1267,22 @@
         <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
@@ -1256,22 +1290,22 @@
         <v>128</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>133</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>133</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
@@ -1279,22 +1313,22 @@
         <v>162</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>165</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>165</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
@@ -1302,22 +1336,22 @@
         <v>140</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>144</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>144</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
@@ -1325,22 +1359,22 @@
         <v>63</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>88</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
@@ -1348,22 +1382,22 @@
         <v>181</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="G6" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
@@ -1371,22 +1405,22 @@
         <v>190</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>278</v>
-      </c>
       <c r="G7" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
@@ -1394,22 +1428,22 @@
         <v>24</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
@@ -1417,22 +1451,22 @@
         <v>41</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>227</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>227</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -1681,7 +1715,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -1691,10 +1725,11 @@
     <col min="5" max="5" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="2" width="25.290714285714284" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -1719,20 +1754,23 @@
       <c r="G1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>246</v>
-      </c>
       <c r="J1" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>130</v>
       </c>
@@ -1743,10 +1781,10 @@
         <v>128</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>27</v>
@@ -1754,17 +1792,20 @@
       <c r="G2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>27</v>
+      <c r="H2" s="4">
+        <v>1</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>248</v>
+      <c r="L2" s="1" t="s">
+        <v>249</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
@@ -1781,7 +1822,7 @@
         <v>92</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>27</v>
@@ -1789,17 +1830,20 @@
       <c r="G3" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="5">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>248</v>
+      <c r="L3" s="1" t="s">
+        <v>249</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
@@ -1807,7 +1851,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>162</v>
@@ -1824,16 +1868,19 @@
       <c r="G4" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="5">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
@@ -1846,10 +1893,10 @@
         <v>140</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>27</v>
@@ -1857,32 +1904,35 @@
       <c r="G5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>181</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>27</v>
@@ -1890,23 +1940,26 @@
       <c r="G6" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="5">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
         <v>235</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>24</v>
@@ -1915,7 +1968,7 @@
         <v>229</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>27</v>
@@ -1923,17 +1976,20 @@
       <c r="G7" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="5">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>255</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>256</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>257</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
@@ -1941,7 +1997,7 @@
         <v>235</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>24</v>
@@ -1950,7 +2006,7 @@
         <v>220</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>29</v>
@@ -1958,25 +2014,28 @@
       <c r="G8" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="5">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>255</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>256</v>
       </c>
+      <c r="L8" s="1" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>24</v>
@@ -1985,7 +2044,7 @@
         <v>229</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>27</v>
@@ -1993,25 +2052,28 @@
       <c r="G9" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>255</v>
-      </c>
       <c r="K9" s="1" t="s">
-        <v>260</v>
+        <v>256</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>261</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>24</v>
@@ -2020,7 +2082,7 @@
         <v>220</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>29</v>
@@ -2028,25 +2090,28 @@
       <c r="G10" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="5">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>255</v>
-      </c>
       <c r="K10" s="1" t="s">
-        <v>260</v>
+        <v>256</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>261</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>41</v>
@@ -2055,7 +2120,7 @@
         <v>221</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>27</v>
@@ -2063,25 +2128,28 @@
       <c r="G11" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>87</v>
+      <c r="H11" s="5">
+        <v>0</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>87</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>255</v>
+        <v>87</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>260</v>
+        <v>256</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>261</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>41</v>
@@ -2090,7 +2158,7 @@
         <v>221</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>29</v>
@@ -2098,17 +2166,20 @@
       <c r="G12" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>87</v>
+      <c r="H12" s="5">
+        <v>0</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>87</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>255</v>
+        <v>87</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>260</v>
+        <v>256</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>261</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
@@ -2116,7 +2187,7 @@
         <v>224</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>41</v>
@@ -2133,23 +2204,26 @@
       <c r="G13" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="5">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
         <v>230</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>24</v>
@@ -2166,16 +2240,19 @@
       <c r="G14" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="5">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="K14" s="1"/>
+      <c r="K14" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="L14" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2784,12 +2861,12 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="2" width="34.71928571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="2" width="29.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>

</xml_diff>